<commit_message>
Regional files added and Research experiment inside docker
</commit_message>
<xml_diff>
--- a/docker/region_data/raw/Central Ostrobothnia.xlsx
+++ b/docker/region_data/raw/Central Ostrobothnia.xlsx
@@ -1,14 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_A421F19A27D297F2BE7BD32DAAE6530D0FDB46BE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D0B9E95-5983-41FD-B9F1-E8F961CEB29D}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="summary" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="GHG emissions" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="emissions and energy" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="other indicators" state="visible" r:id="rId7"/>
+    <sheet name="summary" sheetId="1" r:id="rId1"/>
+    <sheet name="GHG emissions" sheetId="2" r:id="rId2"/>
+    <sheet name="emissions and energy" sheetId="3" r:id="rId3"/>
+    <sheet name="other indicators" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'emissions and energy'!$A$2:$X$54</definedName>
+  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
@@ -280,17 +287,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -654,14 +663,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="30"/>
+  <sheetFormatPr defaultColWidth="30" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -684,7 +693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -701,13 +710,13 @@
         <v>4.3</v>
       </c>
       <c r="F2">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="G2">
         <v>-75.3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -718,7 +727,7 @@
         <v>8.5</v>
       </c>
       <c r="D3">
-        <v>-71.6</v>
+        <v>-71.599999999999994</v>
       </c>
       <c r="E3">
         <v>0.4</v>
@@ -730,7 +739,7 @@
         <v>-71.7</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -738,13 +747,13 @@
         <v>74.8</v>
       </c>
       <c r="C4">
-        <v>39.2</v>
+        <v>39.200000000000003</v>
       </c>
       <c r="D4">
         <v>-47.6</v>
       </c>
       <c r="E4">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="F4">
         <v>0.6</v>
@@ -753,7 +762,7 @@
         <v>-47.6</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -773,10 +782,10 @@
         <v>0.2</v>
       </c>
       <c r="G5">
-        <v>-75.4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+        <v>-75.400000000000006</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -799,7 +808,7 @@
         <v>-35</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -822,7 +831,7 @@
         <v>-62.6</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
@@ -845,7 +854,7 @@
         <v>-12.5</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
@@ -868,7 +877,7 @@
         <v>-25</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>15</v>
       </c>
@@ -879,7 +888,7 @@
         <v>1.8</v>
       </c>
       <c r="D10">
-        <v>-68.6</v>
+        <v>-68.599999999999994</v>
       </c>
       <c r="E10">
         <v>0.1</v>
@@ -888,10 +897,10 @@
         <v>0</v>
       </c>
       <c r="G10">
-        <v>-68.6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>-68.599999999999994</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
@@ -914,12 +923,12 @@
         <v>-22.2</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B12">
-        <v>322.4</v>
+        <v>322.39999999999998</v>
       </c>
       <c r="C12">
         <v>317</v>
@@ -937,7 +946,7 @@
         <v>-1.8</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>18</v>
       </c>
@@ -960,15 +969,15 @@
         <v>-48.5</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B14">
-        <v>17.1</v>
+        <v>17.100000000000001</v>
       </c>
       <c r="C14">
-        <v>8.2</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="D14">
         <v>-52</v>
@@ -983,7 +992,7 @@
         <v>-52.1</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>20</v>
       </c>
@@ -1006,12 +1015,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B16" s="1">
-        <v>1284.4</v>
+        <v>1284.4000000000001</v>
       </c>
       <c r="C16" s="1">
         <v>743.7</v>
@@ -1029,7 +1038,7 @@
         <v>-42.2</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>22</v>
       </c>
@@ -1052,26 +1061,26 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>24</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:V20"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" defaultColWidth="15"/>
+  <sheetFormatPr defaultColWidth="15" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1139,7 +1148,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
@@ -1195,7 +1204,7 @@
         <v>144.5</v>
       </c>
       <c r="S2">
-        <v>157.2</v>
+        <v>157.19999999999999</v>
       </c>
       <c r="T2">
         <v>143.4</v>
@@ -1207,7 +1216,7 @@
         <v>72.7</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1227,7 +1236,7 @@
         <v>32.1</v>
       </c>
       <c r="G3">
-        <v>36.3</v>
+        <v>36.299999999999997</v>
       </c>
       <c r="H3">
         <v>49.1</v>
@@ -1251,7 +1260,7 @@
         <v>23.8</v>
       </c>
       <c r="O3">
-        <v>20.1</v>
+        <v>20.100000000000001</v>
       </c>
       <c r="P3">
         <v>22</v>
@@ -1275,7 +1284,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -1295,10 +1304,10 @@
         <v>84.3</v>
       </c>
       <c r="G4">
-        <v>70.9</v>
+        <v>70.900000000000006</v>
       </c>
       <c r="H4">
-        <v>81.9</v>
+        <v>81.900000000000006</v>
       </c>
       <c r="I4">
         <v>63.8</v>
@@ -1340,10 +1349,10 @@
         <v>45.1</v>
       </c>
       <c r="V4">
-        <v>39.2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+        <v>39.200000000000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -1369,7 +1378,7 @@
         <v>50.6</v>
       </c>
       <c r="I5">
-        <v>37.7</v>
+        <v>37.700000000000003</v>
       </c>
       <c r="J5">
         <v>41.7</v>
@@ -1378,7 +1387,7 @@
         <v>35.4</v>
       </c>
       <c r="L5">
-        <v>35.2</v>
+        <v>35.200000000000003</v>
       </c>
       <c r="M5">
         <v>31.8</v>
@@ -1405,13 +1414,13 @@
         <v>21.1</v>
       </c>
       <c r="U5">
-        <v>17.1</v>
+        <v>17.100000000000001</v>
       </c>
       <c r="V5">
         <v>15.5</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -1455,7 +1464,7 @@
         <v>20.7</v>
       </c>
       <c r="O6">
-        <v>20.4</v>
+        <v>20.399999999999999</v>
       </c>
       <c r="P6">
         <v>18.7</v>
@@ -1464,7 +1473,7 @@
         <v>19</v>
       </c>
       <c r="R6">
-        <v>20.1</v>
+        <v>20.100000000000001</v>
       </c>
       <c r="S6">
         <v>20</v>
@@ -1473,13 +1482,13 @@
         <v>20.2</v>
       </c>
       <c r="U6">
-        <v>19.1</v>
+        <v>19.100000000000001</v>
       </c>
       <c r="V6">
         <v>14.2</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -1535,24 +1544,24 @@
         <v>85.3</v>
       </c>
       <c r="S7">
-        <v>65.1</v>
+        <v>65.099999999999994</v>
       </c>
       <c r="T7">
         <v>65.8</v>
       </c>
       <c r="U7">
-        <v>65.1</v>
+        <v>65.099999999999994</v>
       </c>
       <c r="V7">
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B8">
-        <v>39.7</v>
+        <v>39.700000000000003</v>
       </c>
       <c r="C8">
         <v>41.7</v>
@@ -1582,7 +1591,7 @@
         <v>44.2</v>
       </c>
       <c r="L8">
-        <v>40.8</v>
+        <v>40.799999999999997</v>
       </c>
       <c r="M8">
         <v>44.9</v>
@@ -1597,25 +1606,25 @@
         <v>40.6</v>
       </c>
       <c r="Q8">
-        <v>40.8</v>
+        <v>40.799999999999997</v>
       </c>
       <c r="R8">
-        <v>39.7</v>
+        <v>39.700000000000003</v>
       </c>
       <c r="S8">
-        <v>37.8</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="T8">
         <v>38.1</v>
       </c>
       <c r="U8">
-        <v>36.7</v>
+        <v>36.700000000000003</v>
       </c>
       <c r="V8">
         <v>36.5</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>14</v>
       </c>
@@ -1647,7 +1656,7 @@
         <v>164.5</v>
       </c>
       <c r="K9">
-        <v>162.2</v>
+        <v>162.19999999999999</v>
       </c>
       <c r="L9">
         <v>146.9</v>
@@ -1656,13 +1665,13 @@
         <v>146.6</v>
       </c>
       <c r="N9">
-        <v>163.2</v>
+        <v>163.19999999999999</v>
       </c>
       <c r="O9">
         <v>153.1</v>
       </c>
       <c r="P9">
-        <v>154.7</v>
+        <v>154.69999999999999</v>
       </c>
       <c r="Q9">
         <v>148.6</v>
@@ -1671,7 +1680,7 @@
         <v>140</v>
       </c>
       <c r="S9">
-        <v>135.3</v>
+        <v>135.30000000000001</v>
       </c>
       <c r="T9">
         <v>131.6</v>
@@ -1683,7 +1692,7 @@
         <v>130.4</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>15</v>
       </c>
@@ -1694,7 +1703,7 @@
         <v>5.6</v>
       </c>
       <c r="D10">
-        <v>8.2</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="E10">
         <v>7.8</v>
@@ -1721,10 +1730,10 @@
         <v>5.3</v>
       </c>
       <c r="M10">
-        <v>4.1</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="N10">
-        <v>4.1</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="O10">
         <v>4</v>
@@ -1751,7 +1760,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
@@ -1762,7 +1771,7 @@
         <v>8.4</v>
       </c>
       <c r="D11">
-        <v>9.7</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="E11">
         <v>10.3</v>
@@ -1783,16 +1792,16 @@
         <v>12.8</v>
       </c>
       <c r="K11">
-        <v>10.2</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="L11">
-        <v>8.8</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="M11">
         <v>10</v>
       </c>
       <c r="N11">
-        <v>8.8</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="O11">
         <v>8.6</v>
@@ -1819,7 +1828,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
@@ -1827,7 +1836,7 @@
         <v>308.2</v>
       </c>
       <c r="C12">
-        <v>322.4</v>
+        <v>322.39999999999998</v>
       </c>
       <c r="D12">
         <v>327</v>
@@ -1836,10 +1845,10 @@
         <v>324.2</v>
       </c>
       <c r="F12">
-        <v>323.4</v>
+        <v>323.39999999999998</v>
       </c>
       <c r="G12">
-        <v>318.9</v>
+        <v>318.89999999999998</v>
       </c>
       <c r="H12">
         <v>328.6</v>
@@ -1878,7 +1887,7 @@
         <v>334.7</v>
       </c>
       <c r="T12">
-        <v>319.6</v>
+        <v>319.60000000000002</v>
       </c>
       <c r="U12">
         <v>317</v>
@@ -1887,7 +1896,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>18</v>
       </c>
@@ -1913,13 +1922,13 @@
         <v>37</v>
       </c>
       <c r="I13">
-        <v>36.2</v>
+        <v>36.200000000000003</v>
       </c>
       <c r="J13">
         <v>34.4</v>
       </c>
       <c r="K13">
-        <v>32.7</v>
+        <v>32.700000000000003</v>
       </c>
       <c r="L13">
         <v>30.9</v>
@@ -1955,7 +1964,7 @@
         <v>22.1</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>19</v>
       </c>
@@ -1963,7 +1972,7 @@
         <v>0.7</v>
       </c>
       <c r="C14">
-        <v>17.1</v>
+        <v>17.100000000000001</v>
       </c>
       <c r="D14">
         <v>19.3</v>
@@ -1972,19 +1981,19 @@
         <v>19.7</v>
       </c>
       <c r="F14">
-        <v>20.1</v>
+        <v>20.100000000000001</v>
       </c>
       <c r="G14">
         <v>19.7</v>
       </c>
       <c r="H14">
-        <v>19.1</v>
+        <v>19.100000000000001</v>
       </c>
       <c r="I14">
-        <v>19.6</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="J14">
-        <v>19.9</v>
+        <v>19.899999999999999</v>
       </c>
       <c r="K14">
         <v>19.5</v>
@@ -1993,7 +2002,7 @@
         <v>19.5</v>
       </c>
       <c r="M14">
-        <v>18.1</v>
+        <v>18.100000000000001</v>
       </c>
       <c r="N14">
         <v>16.7</v>
@@ -2014,16 +2023,16 @@
         <v>11.5</v>
       </c>
       <c r="T14">
-        <v>10.2</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="U14">
         <v>9.5</v>
       </c>
       <c r="V14">
-        <v>8.2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
+        <v>8.1999999999999993</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>20</v>
       </c>
@@ -2091,15 +2100,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>46</v>
       </c>
       <c r="B16" s="1">
-        <v>1177.1</v>
+        <v>1177.0999999999999</v>
       </c>
       <c r="C16" s="1">
-        <v>1284.4</v>
+        <v>1284.4000000000001</v>
       </c>
       <c r="D16" s="1">
         <v>1607.7</v>
@@ -2117,7 +2126,7 @@
         <v>1501.2</v>
       </c>
       <c r="I16" s="1">
-        <v>1258.9</v>
+        <v>1258.9000000000001</v>
       </c>
       <c r="J16" s="1">
         <v>1133.5</v>
@@ -2126,7 +2135,7 @@
         <v>1176.2</v>
       </c>
       <c r="L16" s="1">
-        <v>1115.6</v>
+        <v>1115.5999999999999</v>
       </c>
       <c r="M16" s="1">
         <v>1032.2</v>
@@ -2135,10 +2144,10 @@
         <v>1094.5</v>
       </c>
       <c r="O16" s="1">
-        <v>1027.4</v>
+        <v>1027.4000000000001</v>
       </c>
       <c r="P16" s="1">
-        <v>1054.9</v>
+        <v>1054.9000000000001</v>
       </c>
       <c r="Q16" s="1">
         <v>982.9</v>
@@ -2159,7 +2168,7 @@
         <v>743.7</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>47</v>
       </c>
@@ -2185,13 +2194,13 @@
         <v>22</v>
       </c>
       <c r="I17">
-        <v>18.4</v>
+        <v>18.399999999999999</v>
       </c>
       <c r="J17">
         <v>16.5</v>
       </c>
       <c r="K17">
-        <v>17.1</v>
+        <v>17.100000000000001</v>
       </c>
       <c r="L17">
         <v>16.2</v>
@@ -2227,7 +2236,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>22</v>
       </c>
@@ -2295,32 +2304,32 @@
         <v>67723</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>24</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:X98"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="30" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-    </row>
-    <row r="2" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>48</v>
       </c>
@@ -2394,7 +2403,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -2414,7 +2423,7 @@
         <v>38.4</v>
       </c>
       <c r="G3">
-        <v>33.8</v>
+        <v>33.799999999999997</v>
       </c>
       <c r="H3">
         <v>26.4</v>
@@ -2423,13 +2432,13 @@
         <v>28.9</v>
       </c>
       <c r="J3">
-        <v>38.3</v>
+        <v>38.299999999999997</v>
       </c>
       <c r="K3">
         <v>27.2</v>
       </c>
       <c r="L3">
-        <v>20.4</v>
+        <v>20.399999999999999</v>
       </c>
       <c r="M3">
         <v>24.8</v>
@@ -2468,7 +2477,7 @@
         <v>6.3</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -2485,7 +2494,7 @@
         <v>5.6</v>
       </c>
       <c r="F4">
-        <v>9.7</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="G4">
         <v>8.9</v>
@@ -2497,7 +2506,7 @@
         <v>7.6</v>
       </c>
       <c r="J4">
-        <v>9.3</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="K4">
         <v>7.6</v>
@@ -2536,13 +2545,13 @@
         <v>1.8</v>
       </c>
       <c r="W4">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="X4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -2568,7 +2577,7 @@
         <v>34</v>
       </c>
       <c r="I5">
-        <v>36.3</v>
+        <v>36.299999999999997</v>
       </c>
       <c r="J5">
         <v>46.6</v>
@@ -2616,7 +2625,7 @@
         <v>5.9</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
@@ -2648,7 +2657,7 @@
         <v>373.4</v>
       </c>
       <c r="K6">
-        <v>307.4</v>
+        <v>307.39999999999998</v>
       </c>
       <c r="L6">
         <v>212.4</v>
@@ -2672,7 +2681,7 @@
         <v>181.6</v>
       </c>
       <c r="S6">
-        <v>141.3</v>
+        <v>141.30000000000001</v>
       </c>
       <c r="T6">
         <v>117.3</v>
@@ -2690,7 +2699,7 @@
         <v>59.8</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -2740,7 +2749,7 @@
         <v>19.7</v>
       </c>
       <c r="Q7">
-        <v>16.6</v>
+        <v>16.600000000000001</v>
       </c>
       <c r="R7">
         <v>18.2</v>
@@ -2764,7 +2773,7 @@
         <v>7.1</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -2802,7 +2811,7 @@
         <v>1.8</v>
       </c>
       <c r="M8">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="N8">
         <v>1.7</v>
@@ -2826,10 +2835,10 @@
         <v>1</v>
       </c>
       <c r="U8">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="V8">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="W8">
         <v>0.7</v>
@@ -2838,7 +2847,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
@@ -2882,19 +2891,19 @@
         <v>2.5</v>
       </c>
       <c r="O9">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="P9">
         <v>2.5</v>
       </c>
       <c r="Q9">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="R9">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="S9">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="T9">
         <v>1.7</v>
@@ -2912,7 +2921,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
@@ -2938,7 +2947,7 @@
         <v>42.6</v>
       </c>
       <c r="I10">
-        <v>33.8</v>
+        <v>33.799999999999997</v>
       </c>
       <c r="J10">
         <v>38.6</v>
@@ -2986,7 +2995,7 @@
         <v>19.7</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -3060,7 +3069,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
@@ -3080,7 +3089,7 @@
         <v>33.9</v>
       </c>
       <c r="G12">
-        <v>37.2</v>
+        <v>37.200000000000003</v>
       </c>
       <c r="H12">
         <v>33.6</v>
@@ -3098,10 +3107,10 @@
         <v>27.1</v>
       </c>
       <c r="M12">
-        <v>17.9</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="N12">
-        <v>17.4</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="O12">
         <v>20.2</v>
@@ -3128,13 +3137,13 @@
         <v>19</v>
       </c>
       <c r="W12">
-        <v>16.9</v>
+        <v>16.899999999999999</v>
       </c>
       <c r="X12">
         <v>14.9</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>9</v>
       </c>
@@ -3148,13 +3157,13 @@
         <v>7.8</v>
       </c>
       <c r="E13">
-        <v>8.2</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="F13">
         <v>8</v>
       </c>
       <c r="G13">
-        <v>8.8</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="H13">
         <v>7.9</v>
@@ -3163,7 +3172,7 @@
         <v>7.1</v>
       </c>
       <c r="J13">
-        <v>8.7</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="K13">
         <v>6.4</v>
@@ -3172,13 +3181,13 @@
         <v>6.2</v>
       </c>
       <c r="M13">
-        <v>4.4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="N13">
-        <v>4.4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="O13">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="P13">
         <v>6.9</v>
@@ -3196,7 +3205,7 @@
         <v>5.5</v>
       </c>
       <c r="U13">
-        <v>4.9</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="V13">
         <v>5.4</v>
@@ -3208,7 +3217,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>10</v>
       </c>
@@ -3237,7 +3246,7 @@
         <v>29.5</v>
       </c>
       <c r="J14">
-        <v>32.8</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="K14">
         <v>23.4</v>
@@ -3255,10 +3264,10 @@
         <v>18.5</v>
       </c>
       <c r="P14">
-        <v>19.4</v>
+        <v>19.399999999999999</v>
       </c>
       <c r="Q14">
-        <v>18.9</v>
+        <v>18.899999999999999</v>
       </c>
       <c r="R14">
         <v>17.2</v>
@@ -3282,7 +3291,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
@@ -3326,7 +3335,7 @@
         <v>1.2</v>
       </c>
       <c r="O15">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="P15">
         <v>0.9</v>
@@ -3356,7 +3365,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
@@ -3385,7 +3394,7 @@
         <v>14</v>
       </c>
       <c r="J16">
-        <v>16.1</v>
+        <v>16.100000000000001</v>
       </c>
       <c r="K16">
         <v>12.8</v>
@@ -3415,7 +3424,7 @@
         <v>11.4</v>
       </c>
       <c r="T16">
-        <v>10.2</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="U16">
         <v>11.7</v>
@@ -3430,7 +3439,7 @@
         <v>11.3</v>
       </c>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>11</v>
       </c>
@@ -3447,7 +3456,7 @@
         <v>10.1</v>
       </c>
       <c r="F17">
-        <v>9.8</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="G17">
         <v>10.3</v>
@@ -3456,7 +3465,7 @@
         <v>9.4</v>
       </c>
       <c r="I17">
-        <v>9.7</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="J17">
         <v>11.1</v>
@@ -3465,13 +3474,13 @@
         <v>9</v>
       </c>
       <c r="L17">
-        <v>9.8</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="M17">
         <v>9.1</v>
       </c>
       <c r="N17">
-        <v>9.2</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="O17">
         <v>8.6</v>
@@ -3495,7 +3504,7 @@
         <v>9.1</v>
       </c>
       <c r="V17">
-        <v>8.3</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="W17">
         <v>7.8</v>
@@ -3504,7 +3513,7 @@
         <v>7.4</v>
       </c>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>11</v>
       </c>
@@ -3530,7 +3539,7 @@
         <v>12</v>
       </c>
       <c r="I18">
-        <v>10.2</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="J18">
         <v>10.4</v>
@@ -3545,7 +3554,7 @@
         <v>10.1</v>
       </c>
       <c r="N18">
-        <v>9.2</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="O18">
         <v>9.4</v>
@@ -3569,7 +3578,7 @@
         <v>7.5</v>
       </c>
       <c r="V18">
-        <v>8.7</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="W18">
         <v>7.6</v>
@@ -3578,7 +3587,7 @@
         <v>3.4</v>
       </c>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>11</v>
       </c>
@@ -3652,7 +3661,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>12</v>
       </c>
@@ -3714,19 +3723,19 @@
         <v>85.3</v>
       </c>
       <c r="U20">
-        <v>65.1</v>
+        <v>65.099999999999994</v>
       </c>
       <c r="V20">
         <v>65.8</v>
       </c>
       <c r="W20">
-        <v>65.1</v>
+        <v>65.099999999999994</v>
       </c>
       <c r="X20">
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>13</v>
       </c>
@@ -3773,7 +3782,7 @@
         <v>5.4</v>
       </c>
       <c r="P21">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="Q21">
         <v>5.3</v>
@@ -3788,7 +3797,7 @@
         <v>5.4</v>
       </c>
       <c r="U21">
-        <v>4.9</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="V21">
         <v>4.8</v>
@@ -3800,7 +3809,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>13</v>
       </c>
@@ -3862,19 +3871,19 @@
         <v>20.3</v>
       </c>
       <c r="U22">
-        <v>19.6</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="V22">
-        <v>20.4</v>
+        <v>20.399999999999999</v>
       </c>
       <c r="W22">
-        <v>19.4</v>
+        <v>19.399999999999999</v>
       </c>
       <c r="X22">
         <v>18.8</v>
       </c>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>13</v>
       </c>
@@ -3948,7 +3957,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>13</v>
       </c>
@@ -3974,7 +3983,7 @@
         <v>5.8</v>
       </c>
       <c r="I24">
-        <v>8.3</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="J24">
         <v>13</v>
@@ -4010,7 +4019,7 @@
         <v>4.7</v>
       </c>
       <c r="U24">
-        <v>4.6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="V24">
         <v>3.8</v>
@@ -4022,7 +4031,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>13</v>
       </c>
@@ -4096,7 +4105,7 @@
         <v>7.2</v>
       </c>
     </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>14</v>
       </c>
@@ -4155,22 +4164,22 @@
         <v>87.3</v>
       </c>
       <c r="T26">
-        <v>81.4</v>
+        <v>81.400000000000006</v>
       </c>
       <c r="U26">
-        <v>79.6</v>
+        <v>79.599999999999994</v>
       </c>
       <c r="V26">
         <v>75.5</v>
       </c>
       <c r="W26">
-        <v>73.4</v>
+        <v>73.400000000000006</v>
       </c>
       <c r="X26">
         <v>76.2</v>
       </c>
     </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>14</v>
       </c>
@@ -4211,10 +4220,10 @@
         <v>48.3</v>
       </c>
       <c r="N27">
-        <v>40.2</v>
+        <v>40.200000000000003</v>
       </c>
       <c r="O27">
-        <v>40.7</v>
+        <v>40.700000000000003</v>
       </c>
       <c r="P27">
         <v>49.1</v>
@@ -4229,22 +4238,22 @@
         <v>38</v>
       </c>
       <c r="T27">
-        <v>36.8</v>
+        <v>36.799999999999997</v>
       </c>
       <c r="U27">
         <v>35</v>
       </c>
       <c r="V27">
-        <v>34.3</v>
+        <v>34.299999999999997</v>
       </c>
       <c r="W27">
         <v>32.9</v>
       </c>
       <c r="X27">
-        <v>33.8</v>
-      </c>
-    </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.25">
+        <v>33.799999999999997</v>
+      </c>
+    </row>
+    <row r="28" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>14</v>
       </c>
@@ -4267,10 +4276,10 @@
         <v>2.6</v>
       </c>
       <c r="H28">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="I28">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="J28">
         <v>1.8</v>
@@ -4297,7 +4306,7 @@
         <v>2</v>
       </c>
       <c r="R28">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="S28">
         <v>1.9</v>
@@ -4306,7 +4315,7 @@
         <v>1.4</v>
       </c>
       <c r="U28">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="V28">
         <v>1.3</v>
@@ -4318,7 +4327,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>14</v>
       </c>
@@ -4392,7 +4401,7 @@
         <v>12.1</v>
       </c>
     </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>14</v>
       </c>
@@ -4433,7 +4442,7 @@
         <v>5.7</v>
       </c>
       <c r="N30">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="O30">
         <v>4.8</v>
@@ -4466,7 +4475,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>14</v>
       </c>
@@ -4540,7 +4549,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>15</v>
       </c>
@@ -4560,7 +4569,7 @@
         <v>2.5</v>
       </c>
       <c r="G32">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="H32">
         <v>2.5</v>
@@ -4569,7 +4578,7 @@
         <v>2.1</v>
       </c>
       <c r="J32">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="K32">
         <v>2.4</v>
@@ -4578,7 +4587,7 @@
         <v>2.5</v>
       </c>
       <c r="M32">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="N32">
         <v>2.1</v>
@@ -4605,7 +4614,7 @@
         <v>1.6</v>
       </c>
       <c r="V32">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="W32">
         <v>1.2</v>
@@ -4614,7 +4623,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>15</v>
       </c>
@@ -4646,7 +4655,7 @@
         <v>5.7</v>
       </c>
       <c r="K33">
-        <v>4.4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="L33">
         <v>3.1</v>
@@ -4664,7 +4673,7 @@
         <v>2.5</v>
       </c>
       <c r="Q33">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="R33">
         <v>2.6</v>
@@ -4688,7 +4697,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>15</v>
       </c>
@@ -4762,7 +4771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>15</v>
       </c>
@@ -4836,7 +4845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>16</v>
       </c>
@@ -4910,7 +4919,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>16</v>
       </c>
@@ -4984,7 +4993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>16</v>
       </c>
@@ -5031,7 +5040,7 @@
         <v>3.3</v>
       </c>
       <c r="P38">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="Q38">
         <v>2.5</v>
@@ -5052,13 +5061,13 @@
         <v>1.2</v>
       </c>
       <c r="W38">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="X38">
-        <v>1.1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.25">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>16</v>
       </c>
@@ -5132,11 +5141,10 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B40" s="1"/>
       <c r="C40" t="s">
         <v>52</v>
       </c>
@@ -5204,7 +5212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>16</v>
       </c>
@@ -5278,7 +5286,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="42" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>17</v>
       </c>
@@ -5310,7 +5318,7 @@
         <v>128</v>
       </c>
       <c r="K42">
-        <v>128.7</v>
+        <v>128.69999999999999</v>
       </c>
       <c r="L42">
         <v>129.5</v>
@@ -5319,13 +5327,13 @@
         <v>131.5</v>
       </c>
       <c r="N42">
-        <v>133.7</v>
+        <v>133.69999999999999</v>
       </c>
       <c r="O42">
-        <v>135.2</v>
+        <v>135.19999999999999</v>
       </c>
       <c r="P42">
-        <v>135.8</v>
+        <v>135.80000000000001</v>
       </c>
       <c r="Q42">
         <v>134</v>
@@ -5352,7 +5360,7 @@
         <v>119.1</v>
       </c>
     </row>
-    <row r="43" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>17</v>
       </c>
@@ -5426,11 +5434,10 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B44" s="1"/>
       <c r="C44" t="s">
         <v>52</v>
       </c>
@@ -5498,7 +5505,7 @@
         <v>27.6</v>
       </c>
     </row>
-    <row r="45" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>17</v>
       </c>
@@ -5557,10 +5564,10 @@
         <v>1.2</v>
       </c>
       <c r="T45">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="U45">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="V45">
         <v>1</v>
@@ -5572,7 +5579,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>17</v>
       </c>
@@ -5646,7 +5653,7 @@
         <v>99.2</v>
       </c>
     </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>17</v>
       </c>
@@ -5678,10 +5685,10 @@
         <v>22.7</v>
       </c>
       <c r="K47">
-        <v>20.1</v>
+        <v>20.100000000000001</v>
       </c>
       <c r="L47">
-        <v>19.9</v>
+        <v>19.899999999999999</v>
       </c>
       <c r="M47">
         <v>23</v>
@@ -5690,7 +5697,7 @@
         <v>21.8</v>
       </c>
       <c r="O47">
-        <v>19.6</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="P47">
         <v>21.7</v>
@@ -5699,7 +5706,7 @@
         <v>19.8</v>
       </c>
       <c r="R47">
-        <v>20.1</v>
+        <v>20.100000000000001</v>
       </c>
       <c r="S47">
         <v>20.6</v>
@@ -5708,19 +5715,19 @@
         <v>20.2</v>
       </c>
       <c r="U47">
-        <v>20.4</v>
+        <v>20.399999999999999</v>
       </c>
       <c r="V47">
         <v>20.3</v>
       </c>
       <c r="W47">
-        <v>19.9</v>
+        <v>19.899999999999999</v>
       </c>
       <c r="X47">
         <v>20.5</v>
       </c>
     </row>
-    <row r="48" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>17</v>
       </c>
@@ -5737,7 +5744,7 @@
         <v>8.9</v>
       </c>
       <c r="F48">
-        <v>9.2</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="G48">
         <v>9.1</v>
@@ -5749,7 +5756,7 @@
         <v>8.6</v>
       </c>
       <c r="J48">
-        <v>8.8</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="K48">
         <v>9.1</v>
@@ -5764,7 +5771,7 @@
         <v>10</v>
       </c>
       <c r="O48">
-        <v>10.2</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="P48">
         <v>10.1</v>
@@ -5776,10 +5783,10 @@
         <v>10</v>
       </c>
       <c r="S48">
-        <v>9.8</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="T48">
-        <v>9.2</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="U48">
         <v>9</v>
@@ -5794,7 +5801,7 @@
         <v>7.6</v>
       </c>
     </row>
-    <row r="49" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>18</v>
       </c>
@@ -5808,13 +5815,13 @@
         <v>3.5</v>
       </c>
       <c r="E49">
-        <v>4.4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="F49">
         <v>4.8</v>
       </c>
       <c r="G49">
-        <v>4.6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="H49">
         <v>4.2</v>
@@ -5868,7 +5875,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>18</v>
       </c>
@@ -5891,16 +5898,16 @@
         <v>36.9</v>
       </c>
       <c r="H50">
-        <v>35.3</v>
+        <v>35.299999999999997</v>
       </c>
       <c r="I50">
-        <v>33.3</v>
+        <v>33.299999999999997</v>
       </c>
       <c r="J50">
-        <v>33.2</v>
+        <v>33.200000000000003</v>
       </c>
       <c r="K50">
-        <v>32.7</v>
+        <v>32.700000000000003</v>
       </c>
       <c r="L50">
         <v>31.3</v>
@@ -5939,10 +5946,10 @@
         <v>20.5</v>
       </c>
       <c r="X50">
-        <v>20.1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:24" x14ac:dyDescent="0.25">
+        <v>20.100000000000001</v>
+      </c>
+    </row>
+    <row r="51" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>19</v>
       </c>
@@ -5995,7 +6002,7 @@
         <v>2.5</v>
       </c>
       <c r="R51">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="S51">
         <v>2.1</v>
@@ -6016,7 +6023,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="52" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>19</v>
       </c>
@@ -6069,7 +6076,7 @@
         <v>9.6</v>
       </c>
       <c r="R52">
-        <v>9.2</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="S52">
         <v>8.4</v>
@@ -6090,7 +6097,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="53" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>19</v>
       </c>
@@ -6104,13 +6111,13 @@
         <v>0.7</v>
       </c>
       <c r="E53">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="F53">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="G53">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="H53">
         <v>2.5</v>
@@ -6119,7 +6126,7 @@
         <v>2.4</v>
       </c>
       <c r="J53">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="K53">
         <v>2</v>
@@ -6128,10 +6135,10 @@
         <v>2.1</v>
       </c>
       <c r="M53">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="N53">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="O53">
         <v>2.1</v>
@@ -6164,7 +6171,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="54" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:24" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>19</v>
       </c>
@@ -6208,7 +6215,7 @@
         <v>1.2</v>
       </c>
       <c r="O54">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="P54">
         <v>1.2</v>
@@ -6238,13 +6245,12 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B56" s="1"/>
-    </row>
-    <row r="58" spans="1:24" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>48</v>
       </c>
@@ -6318,7 +6324,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="59" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>7</v>
       </c>
@@ -6341,7 +6347,7 @@
         <v>134.4</v>
       </c>
       <c r="H59">
-        <v>135.7</v>
+        <v>135.69999999999999</v>
       </c>
       <c r="I59">
         <v>141</v>
@@ -6356,7 +6362,7 @@
         <v>147.4</v>
       </c>
       <c r="M59">
-        <v>145.7</v>
+        <v>145.69999999999999</v>
       </c>
       <c r="N59">
         <v>144.5</v>
@@ -6365,19 +6371,19 @@
         <v>143.6</v>
       </c>
       <c r="P59">
-        <v>156.2</v>
+        <v>156.19999999999999</v>
       </c>
       <c r="Q59">
-        <v>155.8</v>
+        <v>155.80000000000001</v>
       </c>
       <c r="R59">
-        <v>157.8</v>
+        <v>157.80000000000001</v>
       </c>
       <c r="S59">
-        <v>141.3</v>
+        <v>141.30000000000001</v>
       </c>
       <c r="T59">
-        <v>141.2</v>
+        <v>141.19999999999999</v>
       </c>
       <c r="U59">
         <v>163.6</v>
@@ -6389,10 +6395,10 @@
         <v>157.6</v>
       </c>
       <c r="X59">
-        <v>162.8</v>
-      </c>
-    </row>
-    <row r="60" spans="1:24" x14ac:dyDescent="0.25">
+        <v>162.80000000000001</v>
+      </c>
+    </row>
+    <row r="60" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>7</v>
       </c>
@@ -6409,10 +6415,10 @@
         <v>32.5</v>
       </c>
       <c r="F60">
-        <v>33.8</v>
+        <v>33.799999999999997</v>
       </c>
       <c r="G60">
-        <v>35.2</v>
+        <v>35.200000000000003</v>
       </c>
       <c r="H60">
         <v>36.5</v>
@@ -6445,7 +6451,7 @@
         <v>31.3</v>
       </c>
       <c r="R60">
-        <v>32.7</v>
+        <v>32.700000000000003</v>
       </c>
       <c r="S60">
         <v>33.9</v>
@@ -6466,7 +6472,7 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="61" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>7</v>
       </c>
@@ -6540,7 +6546,7 @@
         <v>150.6</v>
       </c>
     </row>
-    <row r="62" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>7</v>
       </c>
@@ -6614,7 +6620,7 @@
         <v>1538.4</v>
       </c>
     </row>
-    <row r="63" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>8</v>
       </c>
@@ -6628,19 +6634,19 @@
         <v>100.6</v>
       </c>
       <c r="E63">
-        <v>131.3</v>
+        <v>131.30000000000001</v>
       </c>
       <c r="F63">
-        <v>135.2</v>
+        <v>135.19999999999999</v>
       </c>
       <c r="G63">
-        <v>135.2</v>
+        <v>135.19999999999999</v>
       </c>
       <c r="H63">
         <v>134.6</v>
       </c>
       <c r="I63">
-        <v>137.8</v>
+        <v>137.80000000000001</v>
       </c>
       <c r="J63">
         <v>152.6</v>
@@ -6649,7 +6655,7 @@
         <v>131.6</v>
       </c>
       <c r="L63">
-        <v>141.2</v>
+        <v>141.19999999999999</v>
       </c>
       <c r="M63">
         <v>136.9</v>
@@ -6661,16 +6667,16 @@
         <v>133.1</v>
       </c>
       <c r="P63">
-        <v>145.3</v>
+        <v>145.30000000000001</v>
       </c>
       <c r="Q63">
-        <v>143.3</v>
+        <v>143.30000000000001</v>
       </c>
       <c r="R63">
-        <v>142.7</v>
+        <v>142.69999999999999</v>
       </c>
       <c r="S63">
-        <v>138.3</v>
+        <v>138.30000000000001</v>
       </c>
       <c r="T63">
         <v>138</v>
@@ -6682,13 +6688,13 @@
         <v>153.1</v>
       </c>
       <c r="W63">
-        <v>149.7</v>
+        <v>149.69999999999999</v>
       </c>
       <c r="X63">
         <v>154.1</v>
       </c>
     </row>
-    <row r="64" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>8</v>
       </c>
@@ -6702,10 +6708,10 @@
         <v>7.1</v>
       </c>
       <c r="E64">
-        <v>9.8</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="F64">
-        <v>9.7</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="G64">
         <v>10.4</v>
@@ -6762,7 +6768,7 @@
         <v>11.6</v>
       </c>
     </row>
-    <row r="65" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>8</v>
       </c>
@@ -6776,7 +6782,7 @@
         <v>15.1</v>
       </c>
       <c r="E65">
-        <v>18.4</v>
+        <v>18.399999999999999</v>
       </c>
       <c r="F65">
         <v>15.7</v>
@@ -6788,25 +6794,25 @@
         <v>17.2</v>
       </c>
       <c r="I65">
-        <v>17.1</v>
+        <v>17.100000000000001</v>
       </c>
       <c r="J65">
         <v>17.8</v>
       </c>
       <c r="K65">
-        <v>16.9</v>
+        <v>16.899999999999999</v>
       </c>
       <c r="L65">
-        <v>17.4</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="M65">
         <v>17.2</v>
       </c>
       <c r="N65">
-        <v>17.4</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="O65">
-        <v>17.4</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="P65">
         <v>18.3</v>
@@ -6815,7 +6821,7 @@
         <v>18.7</v>
       </c>
       <c r="R65">
-        <v>17.9</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="S65">
         <v>20.7</v>
@@ -6827,7 +6833,7 @@
         <v>20</v>
       </c>
       <c r="V65">
-        <v>18.4</v>
+        <v>18.399999999999999</v>
       </c>
       <c r="W65">
         <v>20.6</v>
@@ -6836,7 +6842,7 @@
         <v>19.3</v>
       </c>
     </row>
-    <row r="66" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>9</v>
       </c>
@@ -6850,16 +6856,16 @@
         <v>131.4</v>
       </c>
       <c r="E66">
-        <v>138.2</v>
+        <v>138.19999999999999</v>
       </c>
       <c r="F66">
-        <v>150.2</v>
+        <v>150.19999999999999</v>
       </c>
       <c r="G66">
         <v>156</v>
       </c>
       <c r="H66">
-        <v>158.8</v>
+        <v>158.80000000000001</v>
       </c>
       <c r="I66">
         <v>166.7</v>
@@ -6910,7 +6916,7 @@
         <v>295.8</v>
       </c>
     </row>
-    <row r="67" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>9</v>
       </c>
@@ -6924,16 +6930,16 @@
         <v>0.8</v>
       </c>
       <c r="E67">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="F67">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="G67">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H67">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="I67">
         <v>1.2</v>
@@ -6966,10 +6972,10 @@
         <v>1.7</v>
       </c>
       <c r="S67">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="T67">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="U67">
         <v>2.6</v>
@@ -6984,7 +6990,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="68" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>9</v>
       </c>
@@ -6995,10 +7001,10 @@
         <v>85</v>
       </c>
       <c r="D68">
-        <v>136.8</v>
+        <v>136.80000000000001</v>
       </c>
       <c r="E68">
-        <v>128.2</v>
+        <v>128.19999999999999</v>
       </c>
       <c r="F68">
         <v>126.2</v>
@@ -7010,7 +7016,7 @@
         <v>126.7</v>
       </c>
       <c r="I68">
-        <v>145.8</v>
+        <v>145.80000000000001</v>
       </c>
       <c r="J68">
         <v>169.6</v>
@@ -7028,10 +7034,10 @@
         <v>141.4</v>
       </c>
       <c r="O68">
-        <v>141.7</v>
+        <v>141.69999999999999</v>
       </c>
       <c r="P68">
-        <v>155.7</v>
+        <v>155.69999999999999</v>
       </c>
       <c r="Q68">
         <v>160.1</v>
@@ -7040,10 +7046,10 @@
         <v>158.4</v>
       </c>
       <c r="S68">
-        <v>161.3</v>
+        <v>161.30000000000001</v>
       </c>
       <c r="T68">
-        <v>142.7</v>
+        <v>142.69999999999999</v>
       </c>
       <c r="U68">
         <v>165.8</v>
@@ -7058,7 +7064,7 @@
         <v>225.5</v>
       </c>
     </row>
-    <row r="69" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>9</v>
       </c>
@@ -7069,7 +7075,7 @@
         <v>85</v>
       </c>
       <c r="D69">
-        <v>37.8</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="E69">
         <v>35.9</v>
@@ -7078,19 +7084,19 @@
         <v>33.4</v>
       </c>
       <c r="G69">
-        <v>33.8</v>
+        <v>33.799999999999997</v>
       </c>
       <c r="H69">
         <v>33</v>
       </c>
       <c r="I69">
-        <v>37.3</v>
+        <v>37.299999999999997</v>
       </c>
       <c r="J69">
         <v>47</v>
       </c>
       <c r="K69">
-        <v>37.3</v>
+        <v>37.299999999999997</v>
       </c>
       <c r="L69">
         <v>41.8</v>
@@ -7102,7 +7108,7 @@
         <v>39.1</v>
       </c>
       <c r="O69">
-        <v>38.3</v>
+        <v>38.299999999999997</v>
       </c>
       <c r="P69">
         <v>44.7</v>
@@ -7132,7 +7138,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>10</v>
       </c>
@@ -7149,10 +7155,10 @@
         <v>163.9</v>
       </c>
       <c r="F70">
-        <v>163.2</v>
+        <v>163.19999999999999</v>
       </c>
       <c r="G70">
-        <v>157.8</v>
+        <v>157.80000000000001</v>
       </c>
       <c r="H70">
         <v>115</v>
@@ -7173,13 +7179,13 @@
         <v>81.3</v>
       </c>
       <c r="N70">
-        <v>79.1</v>
+        <v>79.099999999999994</v>
       </c>
       <c r="O70">
         <v>69.8</v>
       </c>
       <c r="P70">
-        <v>73.1</v>
+        <v>73.099999999999994</v>
       </c>
       <c r="Q70">
         <v>71</v>
@@ -7206,7 +7212,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="71" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>10</v>
       </c>
@@ -7250,7 +7256,7 @@
         <v>4.7</v>
       </c>
       <c r="O71">
-        <v>4.4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="P71">
         <v>3.3</v>
@@ -7277,10 +7283,10 @@
         <v>3.3</v>
       </c>
       <c r="X71">
-        <v>2.3</v>
-      </c>
-    </row>
-    <row r="72" spans="1:24" x14ac:dyDescent="0.25">
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="72" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>10</v>
       </c>
@@ -7291,10 +7297,10 @@
         <v>85</v>
       </c>
       <c r="D72">
-        <v>79.1</v>
+        <v>79.099999999999994</v>
       </c>
       <c r="E72">
-        <v>65.6</v>
+        <v>65.599999999999994</v>
       </c>
       <c r="F72">
         <v>63.1</v>
@@ -7354,7 +7360,7 @@
         <v>45.1</v>
       </c>
     </row>
-    <row r="73" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>11</v>
       </c>
@@ -7365,7 +7371,7 @@
         <v>85</v>
       </c>
       <c r="D73">
-        <v>154.3</v>
+        <v>154.30000000000001</v>
       </c>
       <c r="E73">
         <v>246</v>
@@ -7383,7 +7389,7 @@
         <v>255.5</v>
       </c>
       <c r="J73">
-        <v>290.6</v>
+        <v>290.60000000000002</v>
       </c>
       <c r="K73">
         <v>243.4</v>
@@ -7428,7 +7434,7 @@
         <v>212.4</v>
       </c>
     </row>
-    <row r="74" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>11</v>
       </c>
@@ -7502,7 +7508,7 @@
         <v>57.2</v>
       </c>
     </row>
-    <row r="75" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>11</v>
       </c>
@@ -7525,7 +7531,7 @@
         <v>10.5</v>
       </c>
       <c r="H75">
-        <v>10.2</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="I75">
         <v>12.2</v>
@@ -7561,7 +7567,7 @@
         <v>14.1</v>
       </c>
       <c r="T75">
-        <v>17.9</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="U75">
         <v>20.9</v>
@@ -7576,7 +7582,7 @@
         <v>18.7</v>
       </c>
     </row>
-    <row r="76" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>12</v>
       </c>
@@ -7587,7 +7593,7 @@
         <v>85</v>
       </c>
       <c r="D76">
-        <v>584.8</v>
+        <v>584.79999999999995</v>
       </c>
       <c r="E76">
         <v>921.3</v>
@@ -7602,10 +7608,10 @@
         <v>713.7</v>
       </c>
       <c r="I76">
-        <v>561.7</v>
+        <v>561.70000000000005</v>
       </c>
       <c r="J76">
-        <v>632.2</v>
+        <v>632.20000000000005</v>
       </c>
       <c r="K76">
         <v>447.6</v>
@@ -7650,7 +7656,7 @@
         <v>678.6</v>
       </c>
     </row>
-    <row r="77" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>13</v>
       </c>
@@ -7691,13 +7697,13 @@
         <v>21.1</v>
       </c>
       <c r="N77">
-        <v>20.4</v>
+        <v>20.399999999999999</v>
       </c>
       <c r="O77">
         <v>20.2</v>
       </c>
       <c r="P77">
-        <v>19.4</v>
+        <v>19.399999999999999</v>
       </c>
       <c r="Q77">
         <v>20.2</v>
@@ -7706,16 +7712,16 @@
         <v>19.8</v>
       </c>
       <c r="S77">
-        <v>20.4</v>
+        <v>20.399999999999999</v>
       </c>
       <c r="T77">
         <v>20.2</v>
       </c>
       <c r="U77">
-        <v>18.9</v>
+        <v>18.899999999999999</v>
       </c>
       <c r="V77">
-        <v>19.1</v>
+        <v>19.100000000000001</v>
       </c>
       <c r="W77">
         <v>20.8</v>
@@ -7724,7 +7730,7 @@
         <v>18.8</v>
       </c>
     </row>
-    <row r="78" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>13</v>
       </c>
@@ -7735,10 +7741,10 @@
         <v>85</v>
       </c>
       <c r="D78">
-        <v>70.1</v>
+        <v>70.099999999999994</v>
       </c>
       <c r="E78">
-        <v>78.4</v>
+        <v>78.400000000000006</v>
       </c>
       <c r="F78">
         <v>87.3</v>
@@ -7750,7 +7756,7 @@
         <v>85.3</v>
       </c>
       <c r="I78">
-        <v>81.4</v>
+        <v>81.400000000000006</v>
       </c>
       <c r="J78">
         <v>82.5</v>
@@ -7777,7 +7783,7 @@
         <v>83.1</v>
       </c>
       <c r="R78">
-        <v>78.1</v>
+        <v>78.099999999999994</v>
       </c>
       <c r="S78">
         <v>79.2</v>
@@ -7798,7 +7804,7 @@
         <v>75.3</v>
       </c>
     </row>
-    <row r="79" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>13</v>
       </c>
@@ -7872,7 +7878,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="80" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>13</v>
       </c>
@@ -7922,7 +7928,7 @@
         <v>21.4</v>
       </c>
       <c r="Q80">
-        <v>20.4</v>
+        <v>20.399999999999999</v>
       </c>
       <c r="R80">
         <v>21.3</v>
@@ -7931,7 +7937,7 @@
         <v>19</v>
       </c>
       <c r="T80">
-        <v>17.6</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="U80">
         <v>17.7</v>
@@ -7946,7 +7952,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="81" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>13</v>
       </c>
@@ -8020,7 +8026,7 @@
         <v>28.7</v>
       </c>
     </row>
-    <row r="82" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>14</v>
       </c>
@@ -8094,7 +8100,7 @@
         <v>312.7</v>
       </c>
     </row>
-    <row r="83" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>14</v>
       </c>
@@ -8162,13 +8168,13 @@
         <v>161.1</v>
       </c>
       <c r="W83">
-        <v>150.2</v>
+        <v>150.19999999999999</v>
       </c>
       <c r="X83">
-        <v>151.8</v>
-      </c>
-    </row>
-    <row r="84" spans="1:24" x14ac:dyDescent="0.25">
+        <v>151.80000000000001</v>
+      </c>
+    </row>
+    <row r="84" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>14</v>
       </c>
@@ -8212,7 +8218,7 @@
         <v>10.4</v>
       </c>
       <c r="O84">
-        <v>9.2</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="P84">
         <v>10.4</v>
@@ -8227,13 +8233,13 @@
         <v>10.6</v>
       </c>
       <c r="T84">
-        <v>8.3</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="U84">
         <v>7.2</v>
       </c>
       <c r="V84">
-        <v>8.3</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="W84">
         <v>7.9</v>
@@ -8242,7 +8248,7 @@
         <v>7.7</v>
       </c>
     </row>
-    <row r="85" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>14</v>
       </c>
@@ -8316,7 +8322,7 @@
         <v>53.1</v>
       </c>
     </row>
-    <row r="86" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>14</v>
       </c>
@@ -8348,10 +8354,10 @@
         <v>21</v>
       </c>
       <c r="K86">
-        <v>19.9</v>
+        <v>19.899999999999999</v>
       </c>
       <c r="L86">
-        <v>19.1</v>
+        <v>19.100000000000001</v>
       </c>
       <c r="M86">
         <v>18.3</v>
@@ -8390,7 +8396,7 @@
         <v>24.7</v>
       </c>
     </row>
-    <row r="87" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>14</v>
       </c>
@@ -8464,7 +8470,7 @@
         <v>5.6</v>
       </c>
     </row>
-    <row r="88" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>15</v>
       </c>
@@ -8478,16 +8484,16 @@
         <v>13.1</v>
       </c>
       <c r="E88">
-        <v>8.7</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="F88">
-        <v>9.3</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="G88">
-        <v>8.2</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="H88">
-        <v>9.2</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="I88">
         <v>7.7</v>
@@ -8502,7 +8508,7 @@
         <v>9.4</v>
       </c>
       <c r="M88">
-        <v>8.3</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="N88">
         <v>7.7</v>
@@ -8529,7 +8535,7 @@
         <v>6.3</v>
       </c>
       <c r="V88">
-        <v>4.4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="W88">
         <v>4.5</v>
@@ -8538,7 +8544,7 @@
         <v>3.4</v>
       </c>
     </row>
-    <row r="89" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>15</v>
       </c>
@@ -8552,10 +8558,10 @@
         <v>13</v>
       </c>
       <c r="E89">
-        <v>19.1</v>
+        <v>19.100000000000001</v>
       </c>
       <c r="F89">
-        <v>19.9</v>
+        <v>19.899999999999999</v>
       </c>
       <c r="G89">
         <v>22</v>
@@ -8600,10 +8606,10 @@
         <v>21.1</v>
       </c>
       <c r="U89">
-        <v>20.1</v>
+        <v>20.100000000000001</v>
       </c>
       <c r="V89">
-        <v>16.4</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="W89">
         <v>17.3</v>
@@ -8612,7 +8618,7 @@
         <v>18.8</v>
       </c>
     </row>
-    <row r="90" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>15</v>
       </c>
@@ -8686,7 +8692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>15</v>
       </c>
@@ -8760,7 +8766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>16</v>
       </c>
@@ -8807,16 +8813,16 @@
         <v>5.4</v>
       </c>
       <c r="P92">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="Q92">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="R92">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="S92">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="T92">
         <v>5.9</v>
@@ -8834,7 +8840,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="93" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>16</v>
       </c>
@@ -8908,7 +8914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>16</v>
       </c>
@@ -8925,7 +8931,7 @@
         <v>6.9</v>
       </c>
       <c r="F94">
-        <v>9.8</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="G94">
         <v>12.4</v>
@@ -8973,16 +8979,16 @@
         <v>3.8</v>
       </c>
       <c r="V94">
-        <v>4.6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="W94">
         <v>4</v>
       </c>
       <c r="X94">
-        <v>4.6</v>
-      </c>
-    </row>
-    <row r="95" spans="1:24" x14ac:dyDescent="0.25">
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="95" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>16</v>
       </c>
@@ -8996,7 +9002,7 @@
         <v>13.3</v>
       </c>
       <c r="E95">
-        <v>9.8</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="F95">
         <v>11.5</v>
@@ -9005,7 +9011,7 @@
         <v>11.2</v>
       </c>
       <c r="H95">
-        <v>16.4</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="I95">
         <v>12.3</v>
@@ -9023,7 +9029,7 @@
         <v>14.9</v>
       </c>
       <c r="N95">
-        <v>9.8</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="O95">
         <v>13.5</v>
@@ -9056,11 +9062,10 @@
         <v>12.8</v>
       </c>
     </row>
-    <row r="96" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B96" s="1"/>
       <c r="C96" t="s">
         <v>85</v>
       </c>
@@ -9128,7 +9133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>16</v>
       </c>
@@ -9202,7 +9207,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="98" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>20</v>
       </c>
@@ -9249,7 +9254,7 @@
         <v>52.6</v>
       </c>
       <c r="P98">
-        <v>146.7</v>
+        <v>146.69999999999999</v>
       </c>
       <c r="Q98">
         <v>211.1</v>
@@ -9273,25 +9278,32 @@
         <v>802.7</v>
       </c>
       <c r="X98">
-        <v>1031.6</v>
+        <v>1031.5999999999999</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:X54" xr:uid="{00000000-0001-0000-0200-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Water transport"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30" style="1" customWidth="1"/>
     <col min="2" max="2" width="60" style="1" customWidth="1"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>